<commit_message>
feat: otimizacao de performance, correcao das abas de estoque, paises e diarios, e destaque ativo de canais
</commit_message>
<xml_diff>
--- a/data/meta.xlsx
+++ b/data/meta.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mqhair-my.sharepoint.com/personal/antonio_mello_mqhair_com_br/Documents/Área de Trabalho/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mqhair.sharepoint.com/sites/vls/docs/TI/PROJETOS BI/ANTIGRAVITY/PROJETOS/DASHBOARD_tv/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{243A6331-DC74-4C43-990E-210E7CC7C713}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="8_{243A6331-DC74-4C43-990E-210E7CC7C713}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D225DF7A-22DC-445E-83CC-458B4CABBE31}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0C7A1C59-4877-4F35-9D19-FFE464CF042D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{0C7A1C59-4877-4F35-9D19-FFE464CF042D}"/>
   </bookViews>
   <sheets>
     <sheet name="metas" sheetId="1" r:id="rId1"/>
+    <sheet name="base_setores" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4643" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5352" uniqueCount="152">
   <si>
     <t>CODVEND</t>
   </si>
@@ -349,6 +350,153 @@
   <si>
     <t>TSA PROMOCOES LTDA</t>
   </si>
+  <si>
+    <t>SETOR 2</t>
+  </si>
+  <si>
+    <t>VAREJO ESPECIALIZADO_2</t>
+  </si>
+  <si>
+    <t>CANAL</t>
+  </si>
+  <si>
+    <t>REGIONAL</t>
+  </si>
+  <si>
+    <t>REG. SP</t>
+  </si>
+  <si>
+    <t>GESTOR REGIONAL</t>
+  </si>
+  <si>
+    <t>REG. RJ -MG -ES</t>
+  </si>
+  <si>
+    <t>BEC REPRESENTAÇ</t>
+  </si>
+  <si>
+    <t>REG. SUL</t>
+  </si>
+  <si>
+    <t>REG. NO -ND</t>
+  </si>
+  <si>
+    <t>WENDER PERICLES</t>
+  </si>
+  <si>
+    <t>W N RICCI CIA L</t>
+  </si>
+  <si>
+    <t>A DA SILVA BRUM</t>
+  </si>
+  <si>
+    <t>AND R ANGELITA</t>
+  </si>
+  <si>
+    <t>RICARDO BASILIO</t>
+  </si>
+  <si>
+    <t>EDWARDO CORREIA</t>
+  </si>
+  <si>
+    <t>TOSCANO E CELAN</t>
+  </si>
+  <si>
+    <t>PATY CALIL REPR</t>
+  </si>
+  <si>
+    <t>RIBEIROS SERVIC</t>
+  </si>
+  <si>
+    <t>NUNES COMERCIO</t>
+  </si>
+  <si>
+    <t>REG RJ - MG - ES</t>
+  </si>
+  <si>
+    <t>MARCIO BRENO</t>
+  </si>
+  <si>
+    <t>REG NO - ND</t>
+  </si>
+  <si>
+    <t>MG MELQUISEDEC</t>
+  </si>
+  <si>
+    <t>MARIA BELLA REP</t>
+  </si>
+  <si>
+    <t>JGB BROKER LTDA</t>
+  </si>
+  <si>
+    <t>JW DUARTE COMER</t>
+  </si>
+  <si>
+    <t>W N COMERCIAL L</t>
+  </si>
+  <si>
+    <t>CEIFA REPRESENT</t>
+  </si>
+  <si>
+    <t>HELCIO MOREIRA</t>
+  </si>
+  <si>
+    <t>ANGELA GRACIELE</t>
+  </si>
+  <si>
+    <t>MM REP. DE PROD</t>
+  </si>
+  <si>
+    <t>EJER COMERCIO D</t>
+  </si>
+  <si>
+    <t>CLEYTON TESTE V</t>
+  </si>
+  <si>
+    <t>PALMEIRA REPRES</t>
+  </si>
+  <si>
+    <t>REIALDO REPI</t>
+  </si>
+  <si>
+    <t>ECOMMERCE - MQ</t>
+  </si>
+  <si>
+    <t>ECOMMERCE - PARLUX</t>
+  </si>
+  <si>
+    <t>GUILHERME REPRE</t>
+  </si>
+  <si>
+    <t>ALLAN AGUIAR</t>
+  </si>
+  <si>
+    <t>FRANCIELLE OLIV</t>
+  </si>
+  <si>
+    <t>MILTON REPRESEN</t>
+  </si>
+  <si>
+    <t>BEAUTY FAIR</t>
+  </si>
+  <si>
+    <t>CARREFOUR</t>
+  </si>
+  <si>
+    <t>AMAZON USA</t>
+  </si>
+  <si>
+    <t>ANDREINA CAROLI</t>
+  </si>
+  <si>
+    <t>FERNANDO ANTONI</t>
+  </si>
+  <si>
+    <t>MARKETING</t>
+  </si>
+  <si>
+    <t>FCC COMERCIO EU</t>
+  </si>
 </sst>
 </file>
 
@@ -417,7 +565,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="4" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -435,6 +583,7 @@
     <xf numFmtId="4" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -40922,11 +41071,18 @@
     </row>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="E1325:F1325"/>
-    <mergeCell ref="E1326:F1326"/>
-    <mergeCell ref="E1327:F1327"/>
-    <mergeCell ref="E1376:F1376"/>
-    <mergeCell ref="E1449:F1449"/>
+    <mergeCell ref="E747:F747"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="E46:F46"/>
+    <mergeCell ref="E51:F51"/>
+    <mergeCell ref="E58:F58"/>
+    <mergeCell ref="E92:F92"/>
+    <mergeCell ref="E114:F114"/>
+    <mergeCell ref="E332:F332"/>
+    <mergeCell ref="E740:F740"/>
+    <mergeCell ref="E742:F742"/>
     <mergeCell ref="E1522:F1522"/>
     <mergeCell ref="E773:F773"/>
     <mergeCell ref="E816:F816"/>
@@ -40934,19 +41090,2998 @@
     <mergeCell ref="E1108:F1108"/>
     <mergeCell ref="E1142:F1142"/>
     <mergeCell ref="E1324:F1324"/>
-    <mergeCell ref="E92:F92"/>
-    <mergeCell ref="E114:F114"/>
-    <mergeCell ref="E332:F332"/>
-    <mergeCell ref="E740:F740"/>
-    <mergeCell ref="E742:F742"/>
-    <mergeCell ref="E747:F747"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="E46:F46"/>
-    <mergeCell ref="E51:F51"/>
-    <mergeCell ref="E58:F58"/>
+    <mergeCell ref="E1325:F1325"/>
+    <mergeCell ref="E1326:F1326"/>
+    <mergeCell ref="E1327:F1327"/>
+    <mergeCell ref="E1376:F1376"/>
+    <mergeCell ref="E1449:F1449"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41172D4C-B0E0-4E82-884E-C3CB36C28746}">
+  <dimension ref="A1:G118"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="24.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
+        <v>20256</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
+        <v>17770</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>18119</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>7206</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>3143</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>3233</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>1719</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>2125</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>13867</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>7213</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>20230</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>9939</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>4597</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
+        <v>13728</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
+        <v>18684</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
+        <v>8678</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="1">
+        <v>32767</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="1">
+        <v>17544</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="1">
+        <v>11</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="1">
+        <v>1871</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="1">
+        <v>7220</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="1">
+        <v>3687</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="1">
+        <v>12150</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="1">
+        <v>20806</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="1">
+        <v>129</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="1">
+        <v>15283</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="1">
+        <v>200</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="1">
+        <v>20804</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="1">
+        <v>138</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" s="1">
+        <v>1780</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" s="1">
+        <v>136</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="1">
+        <v>2099</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="1">
+        <v>1645</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="1">
+        <v>20255</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="1">
+        <v>3228</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" s="1">
+        <v>3899</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" s="1">
+        <v>3654</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A39" s="1">
+        <v>126</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G39" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A40" s="1">
+        <v>7231</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A41" s="1">
+        <v>8172</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G41" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A42" s="1">
+        <v>141</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G42" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A43" s="1">
+        <v>3653</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G43" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A44" s="1">
+        <v>2733</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G44" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45" s="1">
+        <v>7233</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G45" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46" s="1">
+        <v>16978</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A47" s="1">
+        <v>7218</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G47" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48" s="1">
+        <v>12896</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G48" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A49" s="1">
+        <v>2175</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F49" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G49" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A50" s="1">
+        <v>122</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F50" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G50" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A51" s="1">
+        <v>13865</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E51" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F51" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G51" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A52" s="1">
+        <v>7232</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F52" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G52" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A53" s="1">
+        <v>4598</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E53" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F53" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G53" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A54" s="1">
+        <v>7212</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G54" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A55" s="1">
+        <v>3059</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G55" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A56" s="1">
+        <v>130</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G56" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A57" s="1">
+        <v>14197</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F57" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G57" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A58" s="1">
+        <v>7219</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F58" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G58" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A59" s="1">
+        <v>134</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G59" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A60" s="1">
+        <v>2136</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F60" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G60" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A61" s="1">
+        <v>7209</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D61" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F61" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G61" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A62" s="1">
+        <v>11690</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E62" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F62" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G62" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A63" s="1">
+        <v>7208</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E63" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F63" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G63" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A64" s="1">
+        <v>7211</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D64" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E64" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F64" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G64" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A65" s="1">
+        <v>18688</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D65" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E65" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F65" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G65" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A66" s="1">
+        <v>7217</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D66" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E66" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F66" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G66" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A67" s="1">
+        <v>13975</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D67" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E67" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F67" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G67" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A68" s="1">
+        <v>1995</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D68" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E68" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F68" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G68" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A69" s="1">
+        <v>142</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D69" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E69" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F69" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G69" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A70" s="1">
+        <v>7205</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D70" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E70" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F70" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G70" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A71" s="1">
+        <v>14</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D71" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E71" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F71" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G71" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A72" s="1">
+        <v>160</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D72" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E72" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F72" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G72" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A73" s="1">
+        <v>3821</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D73" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E73" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F73" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G73" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A74" s="1">
+        <v>7214</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D74" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E74" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F74" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G74" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A75" s="1">
+        <v>7242</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C75" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D75" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E75" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F75" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G75" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A76" s="1">
+        <v>156</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D76" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E76" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F76" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G76" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A77" s="1">
+        <v>155</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D77" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E77" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F77" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G77" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A78" s="1">
+        <v>13700</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="C78" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D78" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E78" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F78" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="G78" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A79" s="1">
+        <v>7195</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C79" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D79" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E79" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F79" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G79" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A80" s="1">
+        <v>7202</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D80" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E80" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F80" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G80" s="1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A81" s="1">
+        <v>2223</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C81" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D81" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E81" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F81" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G81" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A82" s="1">
+        <v>7203</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D82" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E82" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F82" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G82" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A83" s="1">
+        <v>7204</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D83" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E83" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F83" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G83" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A84" s="1">
+        <v>7199</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C84" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D84" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E84" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F84" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G84" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A85" s="1">
+        <v>7196</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C85" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D85" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E85" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F85" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G85" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A86" s="1">
+        <v>2218</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C86" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D86" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E86" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F86" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G86" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A87" s="1">
+        <v>7201</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C87" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D87" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E87" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F87" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G87" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A88" s="1">
+        <v>4113</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D88" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E88" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F88" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G88" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A89" s="1">
+        <v>7095</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C89" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D89" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E89" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F89" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G89" s="1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A90" s="1">
+        <v>7004</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D90" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E90" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F90" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G90" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A91" s="1">
+        <v>131</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="C91" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D91" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E91" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F91" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G91" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A92" s="1">
+        <v>1374</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D92" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E92" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F92" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G92" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A93" s="1">
+        <v>7197</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C93" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D93" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E93" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F93" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G93" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A94" s="1">
+        <v>7200</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C94" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D94" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E94" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F94" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G94" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A95" s="1">
+        <v>7194</v>
+      </c>
+      <c r="B95" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C95" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D95" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E95" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F95" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G95" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A96" s="1">
+        <v>7192</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C96" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D96" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E96" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F96" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G96" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A97" s="1">
+        <v>125</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="C97" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D97" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E97" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F97" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G97" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A98" s="1">
+        <v>7215</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C98" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D98" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E98" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F98" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G98" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A99" s="1">
+        <v>133</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C99" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D99" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E99" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F99" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G99" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A100" s="1">
+        <v>7193</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C100" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D100" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E100" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F100" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G100" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A101" s="1">
+        <v>140</v>
+      </c>
+      <c r="B101" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C101" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D101" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E101" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F101" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G101" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A102" s="1">
+        <v>3119</v>
+      </c>
+      <c r="B102" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C102" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D102" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E102" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F102" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G102" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A103" s="1">
+        <v>2126</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="C103" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D103" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E103" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F103" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G103" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A104" s="1">
+        <v>201</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="C104" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D104" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E104" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F104" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G104" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A105" s="1">
+        <v>7210</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C105" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D105" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E105" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F105" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G105" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A106" s="1">
+        <v>7207</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="C106" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D106" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E106" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F106" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G106" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A107" s="1">
+        <v>300</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C107" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D107" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E107" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F107" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G107" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A108" s="1">
+        <v>166</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C108" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D108" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E108" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F108" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G108" s="1" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A109" s="1">
+        <v>310</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="C109" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D109" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E109" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F109" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G109" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A110" s="1">
+        <v>154</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="C110" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D110" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E110" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F110" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G110" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A111" s="1">
+        <v>146</v>
+      </c>
+      <c r="B111" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C111" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D111" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E111" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F111" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G111" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A112" s="1">
+        <v>287</v>
+      </c>
+      <c r="B112" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="C112" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D112" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E112" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F112" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G112" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A113" s="1">
+        <v>161</v>
+      </c>
+      <c r="B113" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C113" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D113" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E113" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F113" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G113" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A114" s="1">
+        <v>301</v>
+      </c>
+      <c r="B114" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C114" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D114" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E114" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F114" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G114" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A115" s="1">
+        <v>162</v>
+      </c>
+      <c r="B115" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C115" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D115" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E115" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F115" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G115" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A116" s="4">
+        <v>302</v>
+      </c>
+      <c r="B116" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C116" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D116" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E116" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F116" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G116" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A117" s="10">
+        <v>7258</v>
+      </c>
+      <c r="B117" s="17" t="s">
+        <v>102</v>
+      </c>
+      <c r="C117" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D117" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E117" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="F117" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="G117" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A118" s="4">
+        <v>303</v>
+      </c>
+      <c r="B118" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="C118" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D118" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E118" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F118" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G118" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100FEC2A6C01FC35B4C98F27BF80BD61D04" ma:contentTypeVersion="11" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="2907544e106569120cde375d2fd4e02d">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f7088b10-dfe3-4848-b29c-270b315469ff" xmlns:ns3="415d0f87-2af1-4d4c-b68e-7bef43811897" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="da9cd61046fd5c0494a31fe593fa3def" ns2:_="" ns3:_="">
+    <xsd:import namespace="f7088b10-dfe3-4848-b29c-270b315469ff"/>
+    <xsd:import namespace="415d0f87-2af1-4d4c-b68e-7bef43811897"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="f7088b10-dfe3-4848-b29c-270b315469ff" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="12" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="13" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="14" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="16" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Marcações de imagem" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="cab4244d-f499-41b9-8fad-4a9492403ec6" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="18" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="415d0f87-2af1-4d4c-b68e-7bef43811897" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="17" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{4eaaf60e-8694-456d-a452-90d36ffc2d32}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="415d0f87-2af1-4d4c-b68e-7bef43811897">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de Conteúdo"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f7088b10-dfe3-4848-b29c-270b315469ff">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="415d0f87-2af1-4d4c-b68e-7bef43811897" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C93FA2D9-E1CE-4F38-8EC5-96229338282A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="f7088b10-dfe3-4848-b29c-270b315469ff"/>
+    <ds:schemaRef ds:uri="415d0f87-2af1-4d4c-b68e-7bef43811897"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F52D711C-C9E1-4433-AC8E-25CDB359952B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="f7088b10-dfe3-4848-b29c-270b315469ff"/>
+    <ds:schemaRef ds:uri="415d0f87-2af1-4d4c-b68e-7bef43811897"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4B322A1F-1B71-4738-8C18-6BBC27BF7C51}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>